<commit_message>
new launch window graph
</commit_message>
<xml_diff>
--- a/GoingToJupiter/minimum_delta_v_trajectory_by_date.xlsx
+++ b/GoingToJupiter/minimum_delta_v_trajectory_by_date.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:E222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,10 +448,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Transfer time [days]</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Trajectory</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Launch day</t>
         </is>
@@ -464,12 +469,15 @@
       <c r="B2" t="n">
         <v>4014.055087892199</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>2549.197173461811</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="E2" s="3" t="n">
         <v>49660</v>
       </c>
     </row>
@@ -480,12 +488,15 @@
       <c r="B3" t="n">
         <v>4523.892183728227</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
+      <c r="C3" t="n">
+        <v>2147.545541491706</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>49689</v>
       </c>
     </row>
@@ -496,12 +507,15 @@
       <c r="B4" t="n">
         <v>8320.05782540196</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
+      <c r="C4" t="n">
+        <v>1809.792870170805</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>49690</v>
       </c>
     </row>
@@ -512,12 +526,15 @@
       <c r="B5" t="n">
         <v>15733.06231858284</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
+      <c r="C5" t="n">
+        <v>2547.676656267437</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>49691</v>
       </c>
     </row>
@@ -528,12 +545,15 @@
       <c r="B6" t="n">
         <v>2792.099258051032</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="n">
+        <v>2418.694728996602</v>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="E6" s="3" t="n">
         <v>49720</v>
       </c>
     </row>
@@ -544,12 +564,15 @@
       <c r="B7" t="n">
         <v>3892.33910341701</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
+      <c r="C7" t="n">
+        <v>1844.148747400495</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>49721</v>
       </c>
     </row>
@@ -560,12 +583,15 @@
       <c r="B8" t="n">
         <v>3548.383114334327</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
+      <c r="C8" t="n">
+        <v>2165.408933062228</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>49731</v>
       </c>
     </row>
@@ -576,12 +602,15 @@
       <c r="B9" t="n">
         <v>2194.094353055985</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="n">
+        <v>2421.177020672218</v>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="E9" s="3" t="n">
         <v>49749</v>
       </c>
     </row>
@@ -592,12 +621,15 @@
       <c r="B10" t="n">
         <v>4188.738280471291</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
+      <c r="C10" t="n">
+        <v>2147.355498823109</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>49751</v>
       </c>
     </row>
@@ -608,12 +640,15 @@
       <c r="B11" t="n">
         <v>2870.027924414046</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
+      <c r="C11" t="n">
+        <v>2014.283765730962</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>49757</v>
       </c>
     </row>
@@ -624,12 +659,15 @@
       <c r="B12" t="n">
         <v>2158.958570207707</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" t="n">
+        <v>2408.818487025273</v>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="E12" s="3" t="n">
         <v>49761</v>
       </c>
     </row>
@@ -640,12 +678,15 @@
       <c r="B13" t="n">
         <v>6804.731680469064</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n">
+      <c r="C13" t="n">
+        <v>2192.457482160421</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>49780</v>
       </c>
     </row>
@@ -656,12 +697,15 @@
       <c r="B14" t="n">
         <v>2384.103297490123</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" t="n">
+        <v>2381.87425132062</v>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="E14" s="3" t="n">
         <v>49781</v>
       </c>
     </row>
@@ -672,12 +716,15 @@
       <c r="B15" t="n">
         <v>3439.530765537691</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n">
+      <c r="C15" t="n">
+        <v>2150.8566228381</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>49810</v>
       </c>
     </row>
@@ -688,12 +735,15 @@
       <c r="B16" t="n">
         <v>1923.275363787801</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
+      <c r="C16" t="n">
+        <v>2192.151036208945</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>49811</v>
       </c>
     </row>
@@ -704,12 +754,15 @@
       <c r="B17" t="n">
         <v>3425.211385385666</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n">
+      <c r="C17" t="n">
+        <v>1882.657672009366</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>49812</v>
       </c>
     </row>
@@ -720,12 +773,15 @@
       <c r="B18" t="n">
         <v>1685.813591970005</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
+      <c r="C18" t="n">
+        <v>2247.865780317195</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
         <v>49825</v>
       </c>
     </row>
@@ -736,12 +792,15 @@
       <c r="B19" t="n">
         <v>1749.397915201365</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n">
+      <c r="C19" t="n">
+        <v>2259.602661185481</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>49839</v>
       </c>
     </row>
@@ -752,12 +811,15 @@
       <c r="B20" t="n">
         <v>1754.051220948018</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n">
+      <c r="C20" t="n">
+        <v>2268.734154436177</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>49842</v>
       </c>
     </row>
@@ -768,12 +830,15 @@
       <c r="B21" t="n">
         <v>3073.580033918888</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
+      <c r="C21" t="n">
+        <v>2696.115575550588</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>49873</v>
       </c>
     </row>
@@ -784,12 +849,15 @@
       <c r="B22" t="n">
         <v>6218.415188723526</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" t="n">
+        <v>2278.24115398949</v>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="E22" s="3" t="n">
         <v>49902</v>
       </c>
     </row>
@@ -800,12 +868,15 @@
       <c r="B23" t="n">
         <v>5311.268775563029</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
+      <c r="C23" t="n">
+        <v>2659.159209492987</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>49904</v>
       </c>
     </row>
@@ -816,12 +887,15 @@
       <c r="B24" t="n">
         <v>10352.60012788985</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n">
+      <c r="C24" t="n">
+        <v>2221.323010622914</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>49934</v>
       </c>
     </row>
@@ -832,12 +906,15 @@
       <c r="B25" t="n">
         <v>11517.21402762166</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n">
+      <c r="C25" t="n">
+        <v>2106.161208597895</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>49964</v>
       </c>
     </row>
@@ -848,12 +925,15 @@
       <c r="B26" t="n">
         <v>11831.27101635916</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n">
+      <c r="C26" t="n">
+        <v>1932.617816417112</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>49965</v>
       </c>
     </row>
@@ -864,12 +944,15 @@
       <c r="B27" t="n">
         <v>7485.582718456546</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n">
+      <c r="C27" t="n">
+        <v>2172.44536459794</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>49994</v>
       </c>
     </row>
@@ -880,12 +963,15 @@
       <c r="B28" t="n">
         <v>11013.20471000736</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="n">
+      <c r="C28" t="n">
+        <v>1887.323313268829</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
         <v>49995</v>
       </c>
     </row>
@@ -896,12 +982,15 @@
       <c r="B29" t="n">
         <v>7441.556565931416</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n">
+      <c r="C29" t="n">
+        <v>2174.470689458123</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
         <v>50002</v>
       </c>
     </row>
@@ -912,12 +1001,15 @@
       <c r="B30" t="n">
         <v>10531.56442559575</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="n">
+      <c r="C30" t="n">
+        <v>1875.708955842925</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>50005</v>
       </c>
     </row>
@@ -928,12 +1020,15 @@
       <c r="B31" t="n">
         <v>14690.15501630144</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" t="n">
+        <v>2203.12341552909</v>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="E31" s="3" t="n">
         <v>50023</v>
       </c>
     </row>
@@ -944,12 +1039,15 @@
       <c r="B32" t="n">
         <v>12593.87390044965</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n">
+      <c r="C32" t="n">
+        <v>1871.796680734057</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>50026</v>
       </c>
     </row>
@@ -960,12 +1058,15 @@
       <c r="B33" t="n">
         <v>5258.898560609356</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="n">
+      <c r="C33" t="n">
+        <v>2189.646206298512</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
         <v>50044</v>
       </c>
     </row>
@@ -976,12 +1077,15 @@
       <c r="B34" t="n">
         <v>12566.94131364906</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" t="n">
+        <v>2566.345794266159</v>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="E34" s="3" t="n">
         <v>50055</v>
       </c>
     </row>
@@ -992,12 +1096,15 @@
       <c r="B35" t="n">
         <v>5606.03318477464</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="n">
+      <c r="C35" t="n">
+        <v>2209.142463769347</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
         <v>50057</v>
       </c>
     </row>
@@ -1008,12 +1115,15 @@
       <c r="B36" t="n">
         <v>10502.98879667432</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" t="n">
+        <v>2912.530806627877</v>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="E36" s="3" t="n">
         <v>50086</v>
       </c>
     </row>
@@ -1024,12 +1134,15 @@
       <c r="B37" t="n">
         <v>7310.898772067319</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="n">
+      <c r="C37" t="n">
+        <v>1828.005909077775</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
         <v>50087</v>
       </c>
     </row>
@@ -1040,12 +1153,15 @@
       <c r="B38" t="n">
         <v>5903.189955385513</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="n">
+      <c r="C38" t="n">
+        <v>2327.717433949053</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
         <v>50103</v>
       </c>
     </row>
@@ -1056,12 +1172,15 @@
       <c r="B39" t="n">
         <v>4157.216501496716</v>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n">
+      <c r="C39" t="n">
+        <v>2102.094217118578</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
         <v>50110</v>
       </c>
     </row>
@@ -1072,12 +1191,15 @@
       <c r="B40" t="n">
         <v>9367.025662902255</v>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n">
+      <c r="C40" t="n">
+        <v>1897.593923002144</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
         <v>50114</v>
       </c>
     </row>
@@ -1088,12 +1210,15 @@
       <c r="B41" t="n">
         <v>4212.766195050981</v>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="n">
+      <c r="C41" t="n">
+        <v>2198.372332482092</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
         <v>50116</v>
       </c>
     </row>
@@ -1104,12 +1229,15 @@
       <c r="B42" t="n">
         <v>7282.00165318889</v>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="n">
+      <c r="C42" t="n">
+        <v>1933.902771551656</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
         <v>50145</v>
       </c>
     </row>
@@ -1120,12 +1248,15 @@
       <c r="B43" t="n">
         <v>9333.512282055686</v>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n">
+      <c r="C43" t="n">
+        <v>2340.215568356512</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
         <v>50146</v>
       </c>
     </row>
@@ -1136,12 +1267,15 @@
       <c r="B44" t="n">
         <v>8432.632128542213</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" t="n">
+        <v>2829.503091028412</v>
+      </c>
+      <c r="D44" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="E44" s="3" t="n">
         <v>50147</v>
       </c>
     </row>
@@ -1152,12 +1286,15 @@
       <c r="B45" t="n">
         <v>6423.185268220112</v>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="n">
+      <c r="C45" t="n">
+        <v>1941.768095325454</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
         <v>50175</v>
       </c>
     </row>
@@ -1168,12 +1305,15 @@
       <c r="B46" t="n">
         <v>4097.357354962637</v>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="n">
+      <c r="C46" t="n">
+        <v>1790.01084031046</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
         <v>50176</v>
       </c>
     </row>
@@ -1184,12 +1324,15 @@
       <c r="B47" t="n">
         <v>8669.81700802522</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" t="n">
+        <v>2790.23979448662</v>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D47" s="3" t="n">
+      <c r="E47" s="3" t="n">
         <v>50177</v>
       </c>
     </row>
@@ -1200,12 +1343,15 @@
       <c r="B48" t="n">
         <v>2623.484723817457</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="n">
+      <c r="C48" t="n">
+        <v>2242.7733766652</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
         <v>50206</v>
       </c>
     </row>
@@ -1216,12 +1362,15 @@
       <c r="B49" t="n">
         <v>2993.960184637568</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
+      <c r="C49" t="n">
+        <v>1924.94898001043</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
         <v>50209</v>
       </c>
     </row>
@@ -1232,12 +1381,15 @@
       <c r="B50" t="n">
         <v>1904.095767382581</v>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="n">
+      <c r="C50" t="n">
+        <v>2308.295145207988</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
         <v>50236</v>
       </c>
     </row>
@@ -1248,12 +1400,15 @@
       <c r="B51" t="n">
         <v>3176.9239440372</v>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="n">
+      <c r="C51" t="n">
+        <v>2144.099730097068</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n">
         <v>50238</v>
       </c>
     </row>
@@ -1264,12 +1419,15 @@
       <c r="B52" t="n">
         <v>5896.513043619248</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="n">
+      <c r="C52" t="n">
+        <v>1962.10821264015</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
         <v>50247</v>
       </c>
     </row>
@@ -1280,12 +1438,15 @@
       <c r="B53" t="n">
         <v>1612.872369061143</v>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="n">
+      <c r="C53" t="n">
+        <v>2324.356202279828</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
         <v>50266</v>
       </c>
     </row>
@@ -1296,12 +1457,15 @@
       <c r="B54" t="n">
         <v>3929.322283618183</v>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="n">
+      <c r="C54" t="n">
+        <v>2305.072877103079</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
         <v>50269</v>
       </c>
     </row>
@@ -1312,12 +1476,15 @@
       <c r="B55" t="n">
         <v>8639.123786193522</v>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" t="n">
+        <v>2575.685791325593</v>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D55" s="3" t="n">
+      <c r="E55" s="3" t="n">
         <v>50285</v>
       </c>
     </row>
@@ -1328,12 +1495,15 @@
       <c r="B56" t="n">
         <v>1281.140028060378</v>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="n">
+      <c r="C56" t="n">
+        <v>2263.218591481248</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
         <v>50298</v>
       </c>
     </row>
@@ -1344,12 +1514,15 @@
       <c r="B57" t="n">
         <v>1226.643527751176</v>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="n">
+      <c r="C57" t="n">
+        <v>2246.59451785385</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
         <v>50312</v>
       </c>
     </row>
@@ -1360,12 +1533,15 @@
       <c r="B58" t="n">
         <v>4025.626151603145</v>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" t="n">
+        <v>2461.587991409666</v>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="E58" s="3" t="n">
         <v>50328</v>
       </c>
     </row>
@@ -1376,12 +1552,15 @@
       <c r="B59" t="n">
         <v>1304.435073724873</v>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="n">
+      <c r="C59" t="n">
+        <v>2269.400354333155</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
         <v>50330</v>
       </c>
     </row>
@@ -1392,12 +1571,15 @@
       <c r="B60" t="n">
         <v>5489.657222481161</v>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="n">
+      <c r="C60" t="n">
+        <v>1733.562603245736</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
         <v>50331</v>
       </c>
     </row>
@@ -1408,12 +1590,15 @@
       <c r="B61" t="n">
         <v>7433.167367619011</v>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" t="n">
+        <v>2526.645998924158</v>
+      </c>
+      <c r="D61" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n">
+      <c r="E61" s="3" t="n">
         <v>50346</v>
       </c>
     </row>
@@ -1424,12 +1609,15 @@
       <c r="B62" t="n">
         <v>5730.655802558076</v>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="n">
+      <c r="C62" t="n">
+        <v>1887.823034859797</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
         <v>50359</v>
       </c>
     </row>
@@ -1440,12 +1628,15 @@
       <c r="B63" t="n">
         <v>2061.400631155953</v>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="n">
+      <c r="C63" t="n">
+        <v>2076.551135953471</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
         <v>50360</v>
       </c>
     </row>
@@ -1456,12 +1647,15 @@
       <c r="B64" t="n">
         <v>3483.180135969717</v>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="n">
+      <c r="C64" t="n">
+        <v>2297.972682958062</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
         <v>50391</v>
       </c>
     </row>
@@ -1472,12 +1666,15 @@
       <c r="B65" t="n">
         <v>10050.49417410825</v>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="n">
+      <c r="C65" t="n">
+        <v>1866.170420320066</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
         <v>50422</v>
       </c>
     </row>
@@ -1488,12 +1685,15 @@
       <c r="B66" t="n">
         <v>13143.42643058428</v>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="n">
+      <c r="C66" t="n">
+        <v>2136.34057749607</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
         <v>50450</v>
       </c>
     </row>
@@ -1504,12 +1704,15 @@
       <c r="B67" t="n">
         <v>17605.21103145456</v>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="n">
+      <c r="C67" t="n">
+        <v>1472.972774393054</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
         <v>50452</v>
       </c>
     </row>
@@ -1520,12 +1723,15 @@
       <c r="B68" t="n">
         <v>7953.704450992684</v>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" t="n">
+        <v>2313.811109122985</v>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D68" s="3" t="n">
+      <c r="E68" s="3" t="n">
         <v>50479</v>
       </c>
     </row>
@@ -1536,12 +1742,15 @@
       <c r="B69" t="n">
         <v>10374.61620937778</v>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="n">
+      <c r="C69" t="n">
+        <v>2086.714298284358</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
         <v>50480</v>
       </c>
     </row>
@@ -1552,12 +1761,15 @@
       <c r="B70" t="n">
         <v>10691.16272220942</v>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" t="n">
+        <v>2381.751828698761</v>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D70" s="3" t="n">
+      <c r="E70" s="3" t="n">
         <v>50502</v>
       </c>
     </row>
@@ -1568,12 +1780,15 @@
       <c r="B71" t="n">
         <v>9533.710982477673</v>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="n">
+      <c r="C71" t="n">
+        <v>2432.63302981191</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
         <v>50510</v>
       </c>
     </row>
@@ -1584,12 +1799,15 @@
       <c r="B72" t="n">
         <v>10125.14591720093</v>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="n">
+      <c r="C72" t="n">
+        <v>1756.452140534336</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
         <v>50511</v>
       </c>
     </row>
@@ -1600,12 +1818,15 @@
       <c r="B73" t="n">
         <v>9314.139912326753</v>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="n">
+      <c r="C73" t="n">
+        <v>2451.70808029176</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
         <v>50523</v>
       </c>
     </row>
@@ -1616,12 +1837,15 @@
       <c r="B74" t="n">
         <v>9501.685650544772</v>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="n">
+      <c r="C74" t="n">
+        <v>2226.430164437737</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
         <v>50540</v>
       </c>
     </row>
@@ -1632,12 +1856,15 @@
       <c r="B75" t="n">
         <v>11190.77427650684</v>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="n">
+      <c r="C75" t="n">
+        <v>2434.966342797619</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
         <v>50542</v>
       </c>
     </row>
@@ -1648,12 +1875,15 @@
       <c r="B76" t="n">
         <v>8914.921738761195</v>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="n">
+      <c r="C76" t="n">
+        <v>1982.754346460781</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
         <v>50571</v>
       </c>
     </row>
@@ -1664,12 +1894,15 @@
       <c r="B77" t="n">
         <v>4970.409846064256</v>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="n">
+      <c r="C77" t="n">
+        <v>1868.19844205007</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n">
         <v>50572</v>
       </c>
     </row>
@@ -1680,12 +1913,15 @@
       <c r="B78" t="n">
         <v>4926.09731237362</v>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="n">
+      <c r="C78" t="n">
+        <v>1911.973287358774</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n">
         <v>50577</v>
       </c>
     </row>
@@ -1696,12 +1932,15 @@
       <c r="B79" t="n">
         <v>5504.271794751188</v>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="n">
+      <c r="C79" t="n">
+        <v>2285.51146039578</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n">
         <v>50584</v>
       </c>
     </row>
@@ -1712,12 +1951,15 @@
       <c r="B80" t="n">
         <v>7411.010111142448</v>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="n">
+      <c r="C80" t="n">
+        <v>2192.791410556332</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n">
         <v>50601</v>
       </c>
     </row>
@@ -1728,12 +1970,15 @@
       <c r="B81" t="n">
         <v>5419.024794353403</v>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="n">
+      <c r="C81" t="n">
+        <v>2334.570352736235</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="n">
         <v>50603</v>
       </c>
     </row>
@@ -1744,12 +1989,15 @@
       <c r="B82" t="n">
         <v>15592.91114340716</v>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" t="n">
+        <v>2182.623987649073</v>
+      </c>
+      <c r="D82" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D82" s="3" t="n">
+      <c r="E82" s="3" t="n">
         <v>50609</v>
       </c>
     </row>
@@ -1760,12 +2008,15 @@
       <c r="B83" t="n">
         <v>8623.181127884431</v>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="n">
+      <c r="C83" t="n">
+        <v>1979.60111981427</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
         <v>50625</v>
       </c>
     </row>
@@ -1776,12 +2027,15 @@
       <c r="B84" t="n">
         <v>6087.053671843214</v>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="n">
+      <c r="C84" t="n">
+        <v>2154.938259939948</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n">
         <v>50632</v>
       </c>
     </row>
@@ -1792,12 +2046,15 @@
       <c r="B85" t="n">
         <v>8636.15812024055</v>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="n">
+      <c r="C85" t="n">
+        <v>2006.613786012682</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="n">
         <v>50634</v>
       </c>
     </row>
@@ -1808,12 +2065,15 @@
       <c r="B86" t="n">
         <v>10082.12352184699</v>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="n">
+      <c r="C86" t="n">
+        <v>2210.291767919855</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n">
         <v>50662</v>
       </c>
     </row>
@@ -1824,12 +2084,15 @@
       <c r="B87" t="n">
         <v>16317.29067598553</v>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" t="n">
+        <v>2576.497418381885</v>
+      </c>
+      <c r="D87" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D87" s="3" t="n">
+      <c r="E87" s="3" t="n">
         <v>50663</v>
       </c>
     </row>
@@ -1840,12 +2103,15 @@
       <c r="B88" t="n">
         <v>6971.32766144599</v>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="n">
+      <c r="C88" t="n">
+        <v>2656.521348767914</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="n">
         <v>50664</v>
       </c>
     </row>
@@ -1856,12 +2122,15 @@
       <c r="B89" t="n">
         <v>5724.401290286592</v>
       </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="n">
+      <c r="C89" t="n">
+        <v>1855.304974749868</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="n">
         <v>50693</v>
       </c>
     </row>
@@ -1872,12 +2141,15 @@
       <c r="B90" t="n">
         <v>14053.35985024147</v>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" t="n">
+        <v>2510.539464482986</v>
+      </c>
+      <c r="D90" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D90" s="3" t="n">
+      <c r="E90" s="3" t="n">
         <v>50694</v>
       </c>
     </row>
@@ -1888,12 +2160,15 @@
       <c r="B91" t="n">
         <v>8400.739992649806</v>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="n">
+      <c r="C91" t="n">
+        <v>1440.375654276172</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="n">
         <v>50701</v>
       </c>
     </row>
@@ -1904,12 +2179,15 @@
       <c r="B92" t="n">
         <v>8991.286452426157</v>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="n">
+      <c r="C92" t="n">
+        <v>2197.513254430934</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="n">
         <v>50722</v>
       </c>
     </row>
@@ -1920,12 +2198,15 @@
       <c r="B93" t="n">
         <v>8528.383512543847</v>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="n">
+      <c r="C93" t="n">
+        <v>1809.368534275456</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="n">
         <v>50724</v>
       </c>
     </row>
@@ -1936,12 +2217,15 @@
       <c r="B94" t="n">
         <v>8994.47945288652</v>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="n">
+      <c r="C94" t="n">
+        <v>2184.748565254792</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="n">
         <v>50725</v>
       </c>
     </row>
@@ -1952,12 +2236,15 @@
       <c r="B95" t="n">
         <v>8420.998416839837</v>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="n">
+      <c r="C95" t="n">
+        <v>1859.526083568553</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="n">
         <v>50740</v>
       </c>
     </row>
@@ -1968,12 +2255,15 @@
       <c r="B96" t="n">
         <v>7120.708598626936</v>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" t="n">
+        <v>2358.281446849489</v>
+      </c>
+      <c r="D96" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D96" s="3" t="n">
+      <c r="E96" s="3" t="n">
         <v>50754</v>
       </c>
     </row>
@@ -1984,12 +2274,15 @@
       <c r="B97" t="n">
         <v>8450.061692567881</v>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="n">
+      <c r="C97" t="n">
+        <v>1878.852391323249</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="n">
         <v>50756</v>
       </c>
     </row>
@@ -2000,12 +2293,15 @@
       <c r="B98" t="n">
         <v>6423.328891556714</v>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" t="n">
+        <v>2339.467481898279</v>
+      </c>
+      <c r="D98" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D98" s="3" t="n">
+      <c r="E98" s="3" t="n">
         <v>50785</v>
       </c>
     </row>
@@ -2016,12 +2312,15 @@
       <c r="B99" t="n">
         <v>8629.505628092676</v>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D99" s="3" t="n">
+      <c r="C99" t="n">
+        <v>1916.702946955712</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="n">
         <v>50787</v>
       </c>
     </row>
@@ -2032,12 +2331,15 @@
       <c r="B100" t="n">
         <v>8910.971937618671</v>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D100" s="3" t="n">
+      <c r="C100" t="n">
+        <v>1998.110807810896</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="n">
         <v>50815</v>
       </c>
     </row>
@@ -2048,12 +2350,15 @@
       <c r="B101" t="n">
         <v>4325.631370845627</v>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" t="n">
+        <v>2308.635154570006</v>
+      </c>
+      <c r="D101" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D101" s="3" t="n">
+      <c r="E101" s="3" t="n">
         <v>50817</v>
       </c>
     </row>
@@ -2064,12 +2369,15 @@
       <c r="B102" t="n">
         <v>4167.977572363327</v>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" t="n">
+        <v>2294.505975461052</v>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D102" s="3" t="n">
+      <c r="E102" s="3" t="n">
         <v>50835</v>
       </c>
     </row>
@@ -2080,12 +2388,15 @@
       <c r="B103" t="n">
         <v>13786.93976366671</v>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="n">
+      <c r="C103" t="n">
+        <v>1737.000470174526</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n">
         <v>50845</v>
       </c>
     </row>
@@ -2096,12 +2407,15 @@
       <c r="B104" t="n">
         <v>13625.64212755976</v>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="n">
+      <c r="C104" t="n">
+        <v>2607.479208896762</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="n">
         <v>50853</v>
       </c>
     </row>
@@ -2112,12 +2426,15 @@
       <c r="B105" t="n">
         <v>3678.106718036061</v>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="n">
+      <c r="C105" t="n">
+        <v>2058.479935469316</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="n">
         <v>50875</v>
       </c>
     </row>
@@ -2128,12 +2445,15 @@
       <c r="B106" t="n">
         <v>8492.148314168053</v>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="n">
+      <c r="C106" t="n">
+        <v>1761.84468458551</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="n">
         <v>50876</v>
       </c>
     </row>
@@ -2144,12 +2464,15 @@
       <c r="B107" t="n">
         <v>3055.610235271717</v>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="n">
+      <c r="C107" t="n">
+        <v>2127.739365076152</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="n">
         <v>50905</v>
       </c>
     </row>
@@ -2160,12 +2483,15 @@
       <c r="B108" t="n">
         <v>4358.456162985729</v>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="n">
+      <c r="C108" t="n">
+        <v>1797.95349274327</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="n">
         <v>50906</v>
       </c>
     </row>
@@ -2176,12 +2502,15 @@
       <c r="B109" t="n">
         <v>14756.49360791315</v>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="n">
+      <c r="C109" t="n">
+        <v>2513.306697699584</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="n">
         <v>50907</v>
       </c>
     </row>
@@ -2192,12 +2521,15 @@
       <c r="B110" t="n">
         <v>2958.267430990622</v>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D110" s="3" t="n">
+      <c r="C110" t="n">
+        <v>2107.226474707514</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="n">
         <v>50914</v>
       </c>
     </row>
@@ -2208,12 +2540,15 @@
       <c r="B111" t="n">
         <v>3086.75257694494</v>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C111" t="n">
+        <v>2194.507348288722</v>
+      </c>
+      <c r="D111" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D111" s="3" t="n">
+      <c r="E111" s="3" t="n">
         <v>50925</v>
       </c>
     </row>
@@ -2224,12 +2559,15 @@
       <c r="B112" t="n">
         <v>3067.572901237036</v>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="n">
+      <c r="C112" t="n">
+        <v>1849.279973934608</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="n">
         <v>50937</v>
       </c>
     </row>
@@ -2240,12 +2578,15 @@
       <c r="B113" t="n">
         <v>3043.963355083282</v>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="n">
+      <c r="C113" t="n">
+        <v>1865.492957054876</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="n">
         <v>50943</v>
       </c>
     </row>
@@ -2256,12 +2597,15 @@
       <c r="B114" t="n">
         <v>3294.552202643603</v>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D114" s="3" t="n">
+      <c r="C114" t="n">
+        <v>1908.095096532966</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="n">
         <v>50968</v>
       </c>
     </row>
@@ -2272,12 +2616,15 @@
       <c r="B115" t="n">
         <v>2217.618581364153</v>
       </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="n">
+      <c r="C115" t="n">
+        <v>2096.524316736547</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="n">
         <v>50997</v>
       </c>
     </row>
@@ -2288,12 +2635,15 @@
       <c r="B116" t="n">
         <v>4384.749504158795</v>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D116" s="3" t="n">
+      <c r="C116" t="n">
+        <v>1651.155113152701</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="n">
         <v>50999</v>
       </c>
     </row>
@@ -2304,12 +2654,15 @@
       <c r="B117" t="n">
         <v>1970.306025961567</v>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D117" s="3" t="n">
+      <c r="C117" t="n">
+        <v>2147.985921787038</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="n">
         <v>51011</v>
       </c>
     </row>
@@ -2320,12 +2673,15 @@
       <c r="B118" t="n">
         <v>11366.03409128407</v>
       </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D118" s="3" t="n">
+      <c r="C118" t="n">
+        <v>1805.289709263106</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="n">
         <v>51028</v>
       </c>
     </row>
@@ -2336,12 +2692,15 @@
       <c r="B119" t="n">
         <v>2257.433812141382</v>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="n">
+      <c r="C119" t="n">
+        <v>2237.352871344337</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="n">
         <v>51029</v>
       </c>
     </row>
@@ -2352,12 +2711,15 @@
       <c r="B120" t="n">
         <v>7663.33484616197</v>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C120" t="n">
+        <v>2052.915523865457</v>
+      </c>
+      <c r="D120" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D120" s="3" t="n">
+      <c r="E120" s="3" t="n">
         <v>51058</v>
       </c>
     </row>
@@ -2368,12 +2730,15 @@
       <c r="B121" t="n">
         <v>3544.412487819436</v>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="n">
+      <c r="C121" t="n">
+        <v>2645.08074555508</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="n">
         <v>51060</v>
       </c>
     </row>
@@ -2384,12 +2749,15 @@
       <c r="B122" t="n">
         <v>7342.952185329328</v>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C122" t="n">
+        <v>2051.336211315354</v>
+      </c>
+      <c r="D122" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D122" s="3" t="n">
+      <c r="E122" s="3" t="n">
         <v>51069</v>
       </c>
     </row>
@@ -2400,12 +2768,15 @@
       <c r="B123" t="n">
         <v>5657.110791458814</v>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="n">
+      <c r="C123" t="n">
+        <v>2671.03893029319</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="n">
         <v>51090</v>
       </c>
     </row>
@@ -2416,12 +2787,15 @@
       <c r="B124" t="n">
         <v>12147.09815144838</v>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D124" s="3" t="n">
+      <c r="C124" t="n">
+        <v>1484.060331592765</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="n">
         <v>51119</v>
       </c>
     </row>
@@ -2432,12 +2806,15 @@
       <c r="B125" t="n">
         <v>10601.52856780689</v>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="n">
+      <c r="C125" t="n">
+        <v>2255.959917207415</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="n">
         <v>51121</v>
       </c>
     </row>
@@ -2448,12 +2825,15 @@
       <c r="B126" t="n">
         <v>12071.0963142543</v>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D126" s="3" t="n">
+      <c r="C126" t="n">
+        <v>1515.439451014626</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="n">
         <v>51127</v>
       </c>
     </row>
@@ -2464,12 +2844,15 @@
       <c r="B127" t="n">
         <v>10071.22019405535</v>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="n">
+      <c r="C127" t="n">
+        <v>2023.289853973595</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="n">
         <v>51151</v>
       </c>
     </row>
@@ -2480,12 +2863,15 @@
       <c r="B128" t="n">
         <v>11154.48227417286</v>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D128" s="3" t="n">
+      <c r="C128" t="n">
+        <v>1876.041014803024</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="n">
         <v>51152</v>
       </c>
     </row>
@@ -2496,12 +2882,15 @@
       <c r="B129" t="n">
         <v>14368.57004452504</v>
       </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D129" s="3" t="n">
+      <c r="C129" t="n">
+        <v>1263.445915302427</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="n">
         <v>51176</v>
       </c>
     </row>
@@ -2512,12 +2901,15 @@
       <c r="B130" t="n">
         <v>7983.122407120793</v>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D130" s="3" t="n">
+      <c r="C130" t="n">
+        <v>1941.527793650004</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="n">
         <v>51181</v>
       </c>
     </row>
@@ -2528,12 +2920,15 @@
       <c r="B131" t="n">
         <v>5764.511135484176</v>
       </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D131" s="3" t="n">
+      <c r="C131" t="n">
+        <v>1913.464708496148</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="n">
         <v>51206</v>
       </c>
     </row>
@@ -2544,12 +2939,15 @@
       <c r="B132" t="n">
         <v>6838.981769905186</v>
       </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D132" s="3" t="n">
+      <c r="C132" t="n">
+        <v>1715.41481908141</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="n">
         <v>51210</v>
       </c>
     </row>
@@ -2560,12 +2958,15 @@
       <c r="B133" t="n">
         <v>11838.75159857189</v>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="n">
+      <c r="C133" t="n">
+        <v>1872.287025476858</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="n">
         <v>51211</v>
       </c>
     </row>
@@ -2576,12 +2977,15 @@
       <c r="B134" t="n">
         <v>5841.571117616584</v>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="n">
+      <c r="C134" t="n">
+        <v>1914.51759334634</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="n">
         <v>51212</v>
       </c>
     </row>
@@ -2592,12 +2996,15 @@
       <c r="B135" t="n">
         <v>11688.32501834102</v>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D135" s="3" t="n">
+      <c r="C135" t="n">
+        <v>1873.63602175968</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="n">
         <v>51213</v>
       </c>
     </row>
@@ -2608,12 +3015,15 @@
       <c r="B136" t="n">
         <v>6834.030789400924</v>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D136" s="3" t="n">
+      <c r="C136" t="n">
+        <v>1730.046319127933</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="n">
         <v>51215</v>
       </c>
     </row>
@@ -2624,12 +3034,15 @@
       <c r="B137" t="n">
         <v>7048.574004383088</v>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D137" s="3" t="n">
+      <c r="C137" t="n">
+        <v>1875.004604960936</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="n">
         <v>51242</v>
       </c>
     </row>
@@ -2640,12 +3053,15 @@
       <c r="B138" t="n">
         <v>8999.343024112595</v>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C138" t="n">
+        <v>2767.170753541317</v>
+      </c>
+      <c r="D138" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D138" s="3" t="n">
+      <c r="E138" s="3" t="n">
         <v>51271</v>
       </c>
     </row>
@@ -2656,12 +3072,15 @@
       <c r="B139" t="n">
         <v>6160.902376060669</v>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="n">
+      <c r="C139" t="n">
+        <v>2077.232967848855</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="n">
         <v>51272</v>
       </c>
     </row>
@@ -2672,12 +3091,15 @@
       <c r="B140" t="n">
         <v>13802.05950121409</v>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D140" s="3" t="n">
+      <c r="C140" t="n">
+        <v>1753.441528391346</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="n">
         <v>51273</v>
       </c>
     </row>
@@ -2688,12 +3110,15 @@
       <c r="B141" t="n">
         <v>6085.499301724671</v>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="n">
+      <c r="C141" t="n">
+        <v>2056.691656881615</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="n">
         <v>51291</v>
       </c>
     </row>
@@ -2704,12 +3129,15 @@
       <c r="B142" t="n">
         <v>4437.260464211735</v>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D142" s="3" t="n">
+      <c r="C142" t="n">
+        <v>1903.770259245576</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="n">
         <v>51297</v>
       </c>
     </row>
@@ -2720,12 +3148,15 @@
       <c r="B143" t="n">
         <v>7745.327282133348</v>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C143" t="n">
+        <v>2906.838043117208</v>
+      </c>
+      <c r="D143" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D143" s="3" t="n">
+      <c r="E143" s="3" t="n">
         <v>51302</v>
       </c>
     </row>
@@ -2736,12 +3167,15 @@
       <c r="B144" t="n">
         <v>4482.402297961162</v>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D144" s="3" t="n">
+      <c r="C144" t="n">
+        <v>1993.749598666359</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="n">
         <v>51303</v>
       </c>
     </row>
@@ -2752,12 +3186,15 @@
       <c r="B145" t="n">
         <v>7094.944445968797</v>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C145" t="n">
+        <v>2863.615621671772</v>
+      </c>
+      <c r="D145" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D145" s="3" t="n">
+      <c r="E145" s="3" t="n">
         <v>51332</v>
       </c>
     </row>
@@ -2768,12 +3205,15 @@
       <c r="B146" t="n">
         <v>7094.636431274392</v>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C146" t="n">
+        <v>2862.254079842318</v>
+      </c>
+      <c r="D146" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D146" s="3" t="n">
+      <c r="E146" s="3" t="n">
         <v>51334</v>
       </c>
     </row>
@@ -2784,12 +3224,15 @@
       <c r="B147" t="n">
         <v>5911.622384470073</v>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D147" s="3" t="n">
+      <c r="C147" t="n">
+        <v>1819.916866058876</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="n">
         <v>51363</v>
       </c>
     </row>
@@ -2800,12 +3243,15 @@
       <c r="B148" t="n">
         <v>4465.214398931872</v>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D148" s="3" t="n">
+      <c r="C148" t="n">
+        <v>1733.667913607321</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="n">
         <v>51364</v>
       </c>
     </row>
@@ -2816,12 +3262,15 @@
       <c r="B149" t="n">
         <v>3893.471959826318</v>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D149" s="3" t="n">
+      <c r="C149" t="n">
+        <v>1900.715527992519</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="n">
         <v>51382</v>
       </c>
     </row>
@@ -2832,12 +3281,15 @@
       <c r="B150" t="n">
         <v>5430.201724213552</v>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D150" s="3" t="n">
+      <c r="C150" t="n">
+        <v>1824.395794517174</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="n">
         <v>51394</v>
       </c>
     </row>
@@ -2848,12 +3300,15 @@
       <c r="B151" t="n">
         <v>8673.523402327844</v>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D151" s="3" t="n">
+      <c r="C151" t="n">
+        <v>1912.886113091268</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="n">
         <v>51406</v>
       </c>
     </row>
@@ -2864,12 +3319,15 @@
       <c r="B152" t="n">
         <v>4925.629969372643</v>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D152" s="3" t="n">
+      <c r="C152" t="n">
+        <v>1794.353813492281</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="n">
         <v>51424</v>
       </c>
     </row>
@@ -2880,12 +3338,15 @@
       <c r="B153" t="n">
         <v>4838.401851720791</v>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D153" s="3" t="n">
+      <c r="C153" t="n">
+        <v>1497.051854036048</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="n">
         <v>51425</v>
       </c>
     </row>
@@ -2896,12 +3357,15 @@
       <c r="B154" t="n">
         <v>4747.815848525037</v>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D154" s="3" t="n">
+      <c r="C154" t="n">
+        <v>1492.148476618927</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="n">
         <v>51448</v>
       </c>
     </row>
@@ -2912,12 +3376,15 @@
       <c r="B155" t="n">
         <v>6673.66417421671</v>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C155" t="n">
+        <v>3111.483151901069</v>
+      </c>
+      <c r="D155" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D155" s="3" t="n">
+      <c r="E155" s="3" t="n">
         <v>51451</v>
       </c>
     </row>
@@ -2928,12 +3395,15 @@
       <c r="B156" t="n">
         <v>4359.614289158751</v>
       </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D156" s="3" t="n">
+      <c r="C156" t="n">
+        <v>1763.357256622755</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="n">
         <v>51455</v>
       </c>
     </row>
@@ -2944,12 +3414,15 @@
       <c r="B157" t="n">
         <v>6815.264730643279</v>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" t="n">
+        <v>3104.127903474942</v>
+      </c>
+      <c r="D157" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D157" s="3" t="n">
+      <c r="E157" s="3" t="n">
         <v>51456</v>
       </c>
     </row>
@@ -2960,12 +3433,15 @@
       <c r="B158" t="n">
         <v>4206.084386503846</v>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D158" s="3" t="n">
+      <c r="C158" t="n">
+        <v>1760.696471569028</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="n">
         <v>51469</v>
       </c>
     </row>
@@ -2976,12 +3452,15 @@
       <c r="B159" t="n">
         <v>4158.79451060994</v>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D159" s="3" t="n">
+      <c r="C159" t="n">
+        <v>2291.944157574213</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="n">
         <v>51481</v>
       </c>
     </row>
@@ -2992,12 +3471,15 @@
       <c r="B160" t="n">
         <v>7775.376842015268</v>
       </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D160" s="3" t="n">
+      <c r="C160" t="n">
+        <v>1820.303756623213</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="n">
         <v>51485</v>
       </c>
     </row>
@@ -3008,12 +3490,15 @@
       <c r="B161" t="n">
         <v>4402.253579838487</v>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D161" s="3" t="n">
+      <c r="C161" t="n">
+        <v>1794.078508457931</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="n">
         <v>51487</v>
       </c>
     </row>
@@ -3024,12 +3509,15 @@
       <c r="B162" t="n">
         <v>4328.987903602823</v>
       </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D162" s="3" t="n">
+      <c r="C162" t="n">
+        <v>1433.875216269168</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="n">
         <v>51494</v>
       </c>
     </row>
@@ -3040,12 +3528,15 @@
       <c r="B163" t="n">
         <v>4576.852752518196</v>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D163" s="3" t="n">
+      <c r="C163" t="n">
+        <v>1447.981894652621</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="n">
         <v>51518</v>
       </c>
     </row>
@@ -3056,12 +3547,15 @@
       <c r="B164" t="n">
         <v>9091.995045373107</v>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C164" t="n">
+        <v>2497.99240773169</v>
+      </c>
+      <c r="D164" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D164" s="3" t="n">
+      <c r="E164" s="3" t="n">
         <v>51533</v>
       </c>
     </row>
@@ -3072,12 +3566,15 @@
       <c r="B165" t="n">
         <v>6118.997150021129</v>
       </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D165" s="3" t="n">
+      <c r="C165" t="n">
+        <v>1673.359166696871</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="n">
         <v>51546</v>
       </c>
     </row>
@@ -3088,12 +3585,15 @@
       <c r="B166" t="n">
         <v>7687.808394090487</v>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C166" t="n">
+        <v>2987.847521297687</v>
+      </c>
+      <c r="D166" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D166" s="3" t="n">
+      <c r="E166" s="3" t="n">
         <v>51565</v>
       </c>
     </row>
@@ -3104,12 +3604,15 @@
       <c r="B167" t="n">
         <v>6333.644871412651</v>
       </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D167" s="3" t="n">
+      <c r="C167" t="n">
+        <v>2602.662485126461</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="n">
         <v>51577</v>
       </c>
     </row>
@@ -3120,12 +3623,15 @@
       <c r="B168" t="n">
         <v>11174.07466119963</v>
       </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D168" s="3" t="n">
+      <c r="C168" t="n">
+        <v>1727.75762192567</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="n">
         <v>51607</v>
       </c>
     </row>
@@ -3136,12 +3642,15 @@
       <c r="B169" t="n">
         <v>13400.82492276121</v>
       </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D169" s="3" t="n">
+      <c r="C169" t="n">
+        <v>1855.37059417736</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="n">
         <v>51637</v>
       </c>
     </row>
@@ -3152,12 +3661,15 @@
       <c r="B170" t="n">
         <v>14818.16816193844</v>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C170" t="n">
+        <v>2386.592059523776</v>
+      </c>
+      <c r="D170" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D170" s="3" t="n">
+      <c r="E170" s="3" t="n">
         <v>51638</v>
       </c>
     </row>
@@ -3168,12 +3680,15 @@
       <c r="B171" t="n">
         <v>8595.854713828858</v>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D171" s="3" t="n">
+      <c r="C171" t="n">
+        <v>2269.847351243972</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="n">
         <v>51668</v>
       </c>
     </row>
@@ -3184,12 +3699,15 @@
       <c r="B172" t="n">
         <v>8174.799290456387</v>
       </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D172" s="3" t="n">
+      <c r="C172" t="n">
+        <v>2147.048345614171</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="n">
         <v>51676</v>
       </c>
     </row>
@@ -3200,12 +3718,15 @@
       <c r="B173" t="n">
         <v>12589.47391303317</v>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="n">
+      <c r="C173" t="n">
+        <v>1766.874580164999</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="n">
         <v>51697</v>
       </c>
     </row>
@@ -3216,12 +3737,15 @@
       <c r="B174" t="n">
         <v>13244.04560644157</v>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D174" s="3" t="n">
+      <c r="C174" t="n">
+        <v>1253.13956098957</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="n">
         <v>51698</v>
       </c>
     </row>
@@ -3232,12 +3756,15 @@
       <c r="B175" t="n">
         <v>8417.86957078581</v>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D175" s="3" t="n">
+      <c r="C175" t="n">
+        <v>2119.936475248867</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="n">
         <v>51699</v>
       </c>
     </row>
@@ -3248,12 +3775,15 @@
       <c r="B176" t="n">
         <v>10307.17498628802</v>
       </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D176" s="3" t="n">
+      <c r="C176" t="n">
+        <v>1783.731604454192</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="n">
         <v>51728</v>
       </c>
     </row>
@@ -3264,12 +3794,15 @@
       <c r="B177" t="n">
         <v>8386.667339931269</v>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D177" s="3" t="n">
+      <c r="C177" t="n">
+        <v>1694.371215488655</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="n">
         <v>51729</v>
       </c>
     </row>
@@ -3280,12 +3813,15 @@
       <c r="B178" t="n">
         <v>9603.091550642604</v>
       </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D178" s="3" t="n">
+      <c r="C178" t="n">
+        <v>2255.459081668909</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="n">
         <v>51730</v>
       </c>
     </row>
@@ -3296,12 +3832,15 @@
       <c r="B179" t="n">
         <v>11962.03353547625</v>
       </c>
-      <c r="C179" t="inlineStr">
+      <c r="C179" t="n">
+        <v>2576.640101658458</v>
+      </c>
+      <c r="D179" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D179" s="3" t="n">
+      <c r="E179" s="3" t="n">
         <v>51747</v>
       </c>
     </row>
@@ -3312,12 +3851,15 @@
       <c r="B180" t="n">
         <v>9149.5894193731</v>
       </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D180" s="3" t="n">
+      <c r="C180" t="n">
+        <v>1820.616279033955</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="n">
         <v>51759</v>
       </c>
     </row>
@@ -3328,12 +3870,15 @@
       <c r="B181" t="n">
         <v>5217.781460159387</v>
       </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="n">
+      <c r="C181" t="n">
+        <v>1740.323955440265</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="n">
         <v>51760</v>
       </c>
     </row>
@@ -3344,12 +3889,15 @@
       <c r="B182" t="n">
         <v>11955.48384887483</v>
       </c>
-      <c r="C182" t="inlineStr">
+      <c r="C182" t="n">
+        <v>2647.033489853027</v>
+      </c>
+      <c r="D182" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D182" s="3" t="n">
+      <c r="E182" s="3" t="n">
         <v>51761</v>
       </c>
     </row>
@@ -3360,12 +3908,15 @@
       <c r="B183" t="n">
         <v>4959.499203369423</v>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D183" s="3" t="n">
+      <c r="C183" t="n">
+        <v>1841.758754749442</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="n">
         <v>51774</v>
       </c>
     </row>
@@ -3376,12 +3927,15 @@
       <c r="B184" t="n">
         <v>8701.851897132716</v>
       </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D184" s="3" t="n">
+      <c r="C184" t="n">
+        <v>1812.700041785187</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="n">
         <v>51789</v>
       </c>
     </row>
@@ -3392,12 +3946,15 @@
       <c r="B185" t="n">
         <v>5109.841622116415</v>
       </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D185" s="3" t="n">
+      <c r="C185" t="n">
+        <v>2060.588057001461</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="n">
         <v>51791</v>
       </c>
     </row>
@@ -3408,12 +3965,15 @@
       <c r="B186" t="n">
         <v>8632.435231159749</v>
       </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D186" s="3" t="n">
+      <c r="C186" t="n">
+        <v>1928.327733718712</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="n">
         <v>51820</v>
       </c>
     </row>
@@ -3424,12 +3984,15 @@
       <c r="B187" t="n">
         <v>5555.719344187441</v>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D187" s="3" t="n">
+      <c r="C187" t="n">
+        <v>2359.423833415058</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="n">
         <v>51821</v>
       </c>
     </row>
@@ -3440,12 +4003,15 @@
       <c r="B188" t="n">
         <v>8101.327848764682</v>
       </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D188" s="3" t="n">
+      <c r="C188" t="n">
+        <v>1795.13517768021</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="n">
         <v>51836</v>
       </c>
     </row>
@@ -3456,12 +4022,15 @@
       <c r="B189" t="n">
         <v>17947.89344728675</v>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C189" t="n">
+        <v>2180.610321908989</v>
+      </c>
+      <c r="D189" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D189" s="3" t="n">
+      <c r="E189" s="3" t="n">
         <v>51848</v>
       </c>
     </row>
@@ -3472,12 +4041,15 @@
       <c r="B190" t="n">
         <v>8302.85283539742</v>
       </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D190" s="3" t="n">
+      <c r="C190" t="n">
+        <v>1884.475366379848</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="n">
         <v>51850</v>
       </c>
     </row>
@@ -3488,12 +4060,15 @@
       <c r="B191" t="n">
         <v>8172.299834228948</v>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D191" s="3" t="n">
+      <c r="C191" t="n">
+        <v>1793.203126330457</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="n">
         <v>51852</v>
       </c>
     </row>
@@ -3504,12 +4079,15 @@
       <c r="B192" t="n">
         <v>8184.561488697273</v>
       </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D192" s="3" t="n">
+      <c r="C192" t="n">
+        <v>1954.711375936169</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="n">
         <v>51881</v>
       </c>
     </row>
@@ -3520,12 +4098,15 @@
       <c r="B193" t="n">
         <v>6801.565396357986</v>
       </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D193" s="3" t="n">
+      <c r="C193" t="n">
+        <v>2696.224711731692</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="n">
         <v>51883</v>
       </c>
     </row>
@@ -3536,12 +4117,15 @@
       <c r="B194" t="n">
         <v>10690.08752622132</v>
       </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D194" s="3" t="n">
+      <c r="C194" t="n">
+        <v>1346.469347817178</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="n">
         <v>51911</v>
       </c>
     </row>
@@ -3552,12 +4136,15 @@
       <c r="B195" t="n">
         <v>8170.110263856261</v>
       </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D195" s="3" t="n">
+      <c r="C195" t="n">
+        <v>2107.502407154942</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="n">
         <v>51912</v>
       </c>
     </row>
@@ -3568,12 +4155,15 @@
       <c r="B196" t="n">
         <v>9002.132336029576</v>
       </c>
-      <c r="C196" t="inlineStr">
+      <c r="C196" t="n">
+        <v>2404.091572796985</v>
+      </c>
+      <c r="D196" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D196" s="3" t="n">
+      <c r="E196" s="3" t="n">
         <v>51913</v>
       </c>
     </row>
@@ -3584,12 +4174,15 @@
       <c r="B197" t="n">
         <v>7063.264596286135</v>
       </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D197" s="3" t="n">
+      <c r="C197" t="n">
+        <v>1678.720672300867</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="n">
         <v>51940</v>
       </c>
     </row>
@@ -3600,12 +4193,15 @@
       <c r="B198" t="n">
         <v>12732.04175631553</v>
       </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D198" s="3" t="n">
+      <c r="C198" t="n">
+        <v>1873.953440938902</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="n">
         <v>51942</v>
       </c>
     </row>
@@ -3616,12 +4212,15 @@
       <c r="B199" t="n">
         <v>8985.930435077384</v>
       </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="n">
+      <c r="C199" t="n">
+        <v>2154.350767216609</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="n">
         <v>51965</v>
       </c>
     </row>
@@ -3632,12 +4231,15 @@
       <c r="B200" t="n">
         <v>4245.040192377093</v>
       </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D200" s="3" t="n">
+      <c r="C200" t="n">
+        <v>1562.305014415081</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="n">
         <v>51971</v>
       </c>
     </row>
@@ -3648,12 +4250,15 @@
       <c r="B201" t="n">
         <v>8996.077598308617</v>
       </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D201" s="3" t="n">
+      <c r="C201" t="n">
+        <v>2196.026308181693</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="n">
         <v>51972</v>
       </c>
     </row>
@@ -3664,12 +4269,15 @@
       <c r="B202" t="n">
         <v>6602.746473415586</v>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" t="n">
+        <v>2367.993808065424</v>
+      </c>
+      <c r="D202" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D202" s="3" t="n">
+      <c r="E202" s="3" t="n">
         <v>51989</v>
       </c>
     </row>
@@ -3680,12 +4288,15 @@
       <c r="B203" t="n">
         <v>3474.088463728765</v>
       </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D203" s="3" t="n">
+      <c r="C203" t="n">
+        <v>1582.239134339926</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="n">
         <v>52001</v>
       </c>
     </row>
@@ -3696,12 +4307,15 @@
       <c r="B204" t="n">
         <v>5318.997219292112</v>
       </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D204" s="3" t="n">
+      <c r="C204" t="n">
+        <v>2613.025891260736</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="n">
         <v>52026</v>
       </c>
     </row>
@@ -3712,12 +4326,15 @@
       <c r="B205" t="n">
         <v>3281.63139456409</v>
       </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D205" s="3" t="n">
+      <c r="C205" t="n">
+        <v>1616.374875243894</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="n">
         <v>52030</v>
       </c>
     </row>
@@ -3728,12 +4345,15 @@
       <c r="B206" t="n">
         <v>6248.994217109315</v>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C206" t="n">
+        <v>2335.021897195306</v>
+      </c>
+      <c r="D206" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D206" s="3" t="n">
+      <c r="E206" s="3" t="n">
         <v>52032</v>
       </c>
     </row>
@@ -3744,12 +4364,15 @@
       <c r="B207" t="n">
         <v>5460.419012866729</v>
       </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D207" s="3" t="n">
+      <c r="C207" t="n">
+        <v>2607.507344891367</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="n">
         <v>52033</v>
       </c>
     </row>
@@ -3760,12 +4383,15 @@
       <c r="B208" t="n">
         <v>2662.762400757572</v>
       </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D208" s="3" t="n">
+      <c r="C208" t="n">
+        <v>1453.27603483726</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="n">
         <v>52062</v>
       </c>
     </row>
@@ -3776,12 +4402,15 @@
       <c r="B209" t="n">
         <v>12157.68494198515</v>
       </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D209" s="3" t="n">
+      <c r="C209" t="n">
+        <v>1669.099467127853</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="n">
         <v>52063</v>
       </c>
     </row>
@@ -3792,12 +4421,15 @@
       <c r="B210" t="n">
         <v>9589.910969484126</v>
       </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D210" s="3" t="n">
+      <c r="C210" t="n">
+        <v>2594.16229788462</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="n">
         <v>52064</v>
       </c>
     </row>
@@ -3808,12 +4440,15 @@
       <c r="B211" t="n">
         <v>2982.346290770933</v>
       </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D211" s="3" t="n">
+      <c r="C211" t="n">
+        <v>1521.374395463072</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="n">
         <v>52079</v>
       </c>
     </row>
@@ -3824,12 +4459,15 @@
       <c r="B212" t="n">
         <v>5327.966029084346</v>
       </c>
-      <c r="C212" t="inlineStr">
+      <c r="C212" t="n">
+        <v>2263.091849961549</v>
+      </c>
+      <c r="D212" t="inlineStr">
         <is>
           <t>VVEE</t>
         </is>
       </c>
-      <c r="D212" s="3" t="n">
+      <c r="E212" s="3" t="n">
         <v>52091</v>
       </c>
     </row>
@@ -3840,12 +4478,15 @@
       <c r="B213" t="n">
         <v>7060.364129485844</v>
       </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D213" s="3" t="n">
+      <c r="C213" t="n">
+        <v>1690.777989434964</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="n">
         <v>52094</v>
       </c>
     </row>
@@ -3856,12 +4497,15 @@
       <c r="B214" t="n">
         <v>2754.266213292111</v>
       </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D214" s="3" t="n">
+      <c r="C214" t="n">
+        <v>1394.445712241474</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="n">
         <v>52095</v>
       </c>
     </row>
@@ -3872,12 +4516,15 @@
       <c r="B215" t="n">
         <v>4251.892339816433</v>
       </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D215" s="3" t="n">
+      <c r="C215" t="n">
+        <v>1722.473549711632</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="n">
         <v>52125</v>
       </c>
     </row>
@@ -3888,12 +4535,15 @@
       <c r="B216" t="n">
         <v>2876.125446409285</v>
       </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D216" s="3" t="n">
+      <c r="C216" t="n">
+        <v>1420.691732440396</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="n">
         <v>52147</v>
       </c>
     </row>
@@ -3904,12 +4554,15 @@
       <c r="B217" t="n">
         <v>3797.821856234557</v>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D217" s="3" t="n">
+      <c r="C217" t="n">
+        <v>1728.052982365612</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="n">
         <v>52148</v>
       </c>
     </row>
@@ -3920,12 +4573,15 @@
       <c r="B218" t="n">
         <v>2984.841193517434</v>
       </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D218" s="3" t="n">
+      <c r="C218" t="n">
+        <v>1356.671507069931</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="n">
         <v>52156</v>
       </c>
     </row>
@@ -3936,12 +4592,15 @@
       <c r="B219" t="n">
         <v>13974.2104387975</v>
       </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D219" s="3" t="n">
+      <c r="C219" t="n">
+        <v>1708.923615653014</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="n">
         <v>52185</v>
       </c>
     </row>
@@ -3952,12 +4611,15 @@
       <c r="B220" t="n">
         <v>4871.403299368685</v>
       </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>VE</t>
-        </is>
-      </c>
-      <c r="D220" s="3" t="n">
+      <c r="C220" t="n">
+        <v>1744.167896890056</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="n">
         <v>52186</v>
       </c>
     </row>
@@ -3968,12 +4630,15 @@
       <c r="B221" t="n">
         <v>13765.57767700441</v>
       </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>VEE</t>
-        </is>
-      </c>
-      <c r="D221" s="3" t="n">
+      <c r="C221" t="n">
+        <v>1733.507453040056</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>VEE</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="n">
         <v>52201</v>
       </c>
     </row>
@@ -3984,12 +4649,15 @@
       <c r="B222" t="n">
         <v>2398.934475802898</v>
       </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>VVE</t>
-        </is>
-      </c>
-      <c r="D222" s="3" t="n">
+      <c r="C222" t="n">
+        <v>2120.004128953637</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>VVE</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="n">
         <v>52213</v>
       </c>
     </row>

</xml_diff>